<commit_message>
Apply CropX System->Platform wording fix to static block library; update redirect/comparison reports
</commit_message>
<xml_diff>
--- a/cropx-com-sitemap-redirects.xlsx
+++ b/cropx-com-sitemap-redirects.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/laurenhostetter/Documents/github/cropx-website-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CA03B7B-CB86-A54C-857B-305343DC3FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16DDE196-5B57-F949-BAE0-04BC688A74C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5380" yWindow="1480" windowWidth="29420" windowHeight="24280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21000" yWindow="780" windowWidth="20120" windowHeight="24280" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="417">
   <si>
     <t>CropX.com Sitemap Inventory</t>
   </si>
@@ -1228,9 +1228,6 @@
     <t>https://cropx.com/cropx-appoints-john-gates-as-chief-revenue-officer/</t>
   </si>
   <si>
-    <t>reinke-and-cropx-take-partnership-to-next-level-with-unified-platform-integration</t>
-  </si>
-  <si>
     <t>UPDATE REDIRECT</t>
   </si>
   <si>
@@ -1246,9 +1243,6 @@
     <t>https://cropx.com/is-effluent-irrigation-right-for-you/</t>
   </si>
   <si>
-    <t>https://cropx.com//data-helps-farmers-to-get-a-better-understanding-of-the-soil/</t>
-  </si>
-  <si>
     <t>https://cropx.com/proman-partners-with-cropx-to-invest-in-cutting-edge-technology-to-make-farming-more-sustainable/</t>
   </si>
   <si>
@@ -1273,7 +1267,16 @@
     <t>https://cropx.com/cropx-technologies-helps-farmers-understand-pending-nitrogen-regulations/</t>
   </si>
   <si>
-    <t>FIX redirect</t>
+    <t>https://cropx.com/nitrogen-sensing/</t>
+  </si>
+  <si>
+    <t>https://cropx.com/es/knowledge-hub/brochures/</t>
+  </si>
+  <si>
+    <t>https://cropx.com/knowledge-hub/brochures/#hardware-installation</t>
+  </si>
+  <si>
+    <t>https://cropx.com/data-helps-farmers-to-get-a-better-understanding-of-the-soil/</t>
   </si>
 </sst>
 </file>
@@ -1336,7 +1339,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1347,12 +1350,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF243565"/>
         <bgColor rgb="FF243565"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -1411,7 +1408,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1420,23 +1417,20 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1817,17 +1811,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="63" customWidth="1"/>
     <col min="3" max="3" width="0.1640625" customWidth="1"/>
-    <col min="4" max="4" width="21.5" customWidth="1"/>
-    <col min="5" max="5" width="86" customWidth="1"/>
+    <col min="4" max="4" width="86" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>9</v>
       </c>
@@ -1837,11 +1830,11 @@
       <c r="C1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1851,14 +1844,14 @@
       <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="D2" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F2" t="s">
+      <c r="E2" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1868,14 +1861,14 @@
       <c r="C3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="D3" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="F3" t="s">
+      <c r="E3" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1885,14 +1878,14 @@
       <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="D4" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="F4" t="s">
+      <c r="E4" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1902,14 +1895,14 @@
       <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="D5" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="F5" t="s">
+      <c r="E5" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1919,14 +1912,14 @@
       <c r="C6" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="D6" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="F6" t="s">
+      <c r="E6" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1936,14 +1929,14 @@
       <c r="C7" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="D7" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="F7" t="s">
+      <c r="E7" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1953,14 +1946,14 @@
       <c r="C8" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="D8" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F8" t="s">
+      <c r="E8" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1970,14 +1963,14 @@
       <c r="C9" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="D9" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F9" t="s">
+      <c r="E9" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1987,14 +1980,14 @@
       <c r="C10" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="D10" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F10" t="s">
+      <c r="E10" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2004,14 +1997,14 @@
       <c r="C11" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="D11" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F11" t="s">
+      <c r="E11" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2021,14 +2014,14 @@
       <c r="C12" t="s">
         <v>23</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="D12" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F12" t="s">
+      <c r="E12" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2038,14 +2031,14 @@
       <c r="C13" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="D13" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="F13" t="s">
+      <c r="E13" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2055,14 +2048,14 @@
       <c r="C14" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="D14" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F14" t="s">
+      <c r="E14" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2072,14 +2065,14 @@
       <c r="C15" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="D15" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F15" t="s">
+      <c r="E15" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2089,14 +2082,14 @@
       <c r="C16" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="D16" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F16" t="s">
+      <c r="E16" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2106,14 +2099,14 @@
       <c r="C17" t="s">
         <v>35</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="D17" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="E17" s="6" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2123,14 +2116,14 @@
       <c r="C18" t="s">
         <v>35</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="D18" s="10" t="s">
         <v>308</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2140,14 +2133,14 @@
       <c r="C19" t="s">
         <v>35</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="D19" s="10" t="s">
         <v>307</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="E19" s="6" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2157,14 +2150,14 @@
       <c r="C20" t="s">
         <v>35</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="D20" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="E20" s="6" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2174,29 +2167,31 @@
       <c r="C21" t="s">
         <v>40</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="D21" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="5" t="s">
         <v>41</v>
       </c>
       <c r="C22" t="s">
         <v>42</v>
       </c>
-      <c r="E22" s="9"/>
-      <c r="F22" t="s">
+      <c r="D22" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="E22" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2206,14 +2201,14 @@
       <c r="C23" t="s">
         <v>44</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="D23" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="E23" s="6" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2223,14 +2218,14 @@
       <c r="C24" t="s">
         <v>46</v>
       </c>
-      <c r="E24" s="12" t="s">
+      <c r="D24" s="10" t="s">
         <v>295</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="E24" s="6" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2240,14 +2235,14 @@
       <c r="C25" t="s">
         <v>48</v>
       </c>
-      <c r="E25" s="12" t="s">
+      <c r="D25" s="10" t="s">
         <v>314</v>
       </c>
-      <c r="F25" s="6" t="s">
+      <c r="E25" s="6" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2257,14 +2252,14 @@
       <c r="C26" t="s">
         <v>48</v>
       </c>
-      <c r="E26" s="12" t="s">
+      <c r="D26" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="E26" s="6" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2274,14 +2269,14 @@
       <c r="C27" t="s">
         <v>51</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="D27" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F27" t="s">
+      <c r="E27" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2291,14 +2286,14 @@
       <c r="C28" t="s">
         <v>53</v>
       </c>
-      <c r="E28" s="10" t="s">
+      <c r="D28" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F28" t="s">
+      <c r="E28" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2308,14 +2303,14 @@
       <c r="C29" t="s">
         <v>55</v>
       </c>
-      <c r="E29" s="12" t="s">
+      <c r="D29" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="F29" t="s">
+      <c r="E29" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2325,14 +2320,14 @@
       <c r="C30" t="s">
         <v>57</v>
       </c>
-      <c r="E30" s="12" t="s">
+      <c r="D30" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="F30" t="s">
+      <c r="E30" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2342,14 +2337,14 @@
       <c r="C31" t="s">
         <v>59</v>
       </c>
-      <c r="E31" s="12" t="s">
+      <c r="D31" s="10" t="s">
         <v>286</v>
       </c>
-      <c r="F31" t="s">
+      <c r="E31" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2359,14 +2354,14 @@
       <c r="C32" t="s">
         <v>61</v>
       </c>
-      <c r="E32" s="10" t="s">
+      <c r="D32" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F32" t="s">
+      <c r="E32" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2376,12 +2371,14 @@
       <c r="C33" t="s">
         <v>63</v>
       </c>
-      <c r="E33" s="9"/>
-      <c r="F33" t="s">
+      <c r="D33" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="E33" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2391,14 +2388,14 @@
       <c r="C34" t="s">
         <v>65</v>
       </c>
-      <c r="E34" s="12" t="s">
+      <c r="D34" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="F34" s="6" t="s">
+      <c r="E34" s="6" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2408,14 +2405,14 @@
       <c r="C35" t="s">
         <v>67</v>
       </c>
-      <c r="E35" s="12" t="s">
+      <c r="D35" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="E35" s="6" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2425,12 +2422,14 @@
       <c r="C36" t="s">
         <v>69</v>
       </c>
-      <c r="E36" s="9"/>
-      <c r="F36" t="s">
+      <c r="D36" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E36" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2440,14 +2439,14 @@
       <c r="C37" t="s">
         <v>71</v>
       </c>
-      <c r="E37" s="10" t="s">
+      <c r="D37" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F37" t="s">
+      <c r="E37" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2457,14 +2456,14 @@
       <c r="C38" t="s">
         <v>73</v>
       </c>
-      <c r="E38" s="10" t="s">
+      <c r="D38" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F38" t="s">
+      <c r="E38" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2474,14 +2473,14 @@
       <c r="C39" t="s">
         <v>75</v>
       </c>
-      <c r="E39" s="11" t="s">
+      <c r="D39" s="9" t="s">
         <v>291</v>
       </c>
-      <c r="F39" t="s">
+      <c r="E39" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2491,14 +2490,14 @@
       <c r="C40" t="s">
         <v>77</v>
       </c>
-      <c r="E40" s="10" t="s">
+      <c r="D40" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F40" t="s">
+      <c r="E40" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2508,14 +2507,14 @@
       <c r="C41" t="s">
         <v>77</v>
       </c>
-      <c r="E41" s="12" t="s">
+      <c r="D41" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="F41" t="s">
+      <c r="E41" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2525,14 +2524,14 @@
       <c r="C42" t="s">
         <v>80</v>
       </c>
-      <c r="E42" s="12" t="s">
+      <c r="D42" s="10" t="s">
         <v>290</v>
       </c>
-      <c r="F42" t="s">
+      <c r="E42" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2542,14 +2541,14 @@
       <c r="C43" t="s">
         <v>82</v>
       </c>
-      <c r="E43" s="12" t="s">
+      <c r="D43" s="10" t="s">
         <v>314</v>
       </c>
-      <c r="F43" t="s">
+      <c r="E43" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2559,12 +2558,14 @@
       <c r="C44" t="s">
         <v>84</v>
       </c>
-      <c r="E44" s="8"/>
-      <c r="F44" t="s">
+      <c r="D44" s="10" t="s">
+        <v>414</v>
+      </c>
+      <c r="E44" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2574,14 +2575,14 @@
       <c r="C45" t="s">
         <v>86</v>
       </c>
-      <c r="E45" s="12" t="s">
+      <c r="D45" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="F45" t="s">
+      <c r="E45" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2591,14 +2592,14 @@
       <c r="C46" t="s">
         <v>88</v>
       </c>
-      <c r="E46" s="12" t="s">
+      <c r="D46" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="F46" t="s">
+      <c r="E46" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2608,14 +2609,14 @@
       <c r="C47" t="s">
         <v>90</v>
       </c>
-      <c r="E47" s="12" t="s">
+      <c r="D47" s="10" t="s">
         <v>310</v>
       </c>
-      <c r="F47" t="s">
+      <c r="E47" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2625,14 +2626,14 @@
       <c r="C48" t="s">
         <v>92</v>
       </c>
-      <c r="E48" s="12" t="s">
+      <c r="D48" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="F48" t="s">
+      <c r="E48" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2642,14 +2643,14 @@
       <c r="C49" t="s">
         <v>94</v>
       </c>
-      <c r="E49" s="12" t="s">
+      <c r="D49" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="F49" t="s">
+      <c r="E49" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2659,40 +2660,40 @@
       <c r="C50" t="s">
         <v>96</v>
       </c>
-      <c r="E50" s="10" t="s">
+      <c r="D50" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="F50" t="s">
+      <c r="E50" t="s">
         <v>311</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E34" r:id="rId1" xr:uid="{0B8A3AF7-D237-4646-863B-45A17C76C064}"/>
-    <hyperlink ref="E6" r:id="rId2" xr:uid="{654AF1A4-2B50-544D-B5F0-C2CF9018D901}"/>
+    <hyperlink ref="D34" r:id="rId1" xr:uid="{0B8A3AF7-D237-4646-863B-45A17C76C064}"/>
+    <hyperlink ref="D6" r:id="rId2" xr:uid="{654AF1A4-2B50-544D-B5F0-C2CF9018D901}"/>
     <hyperlink ref="B25" r:id="rId3" xr:uid="{43134D95-8BD5-6E4F-9FEE-DD52F933D5DF}"/>
     <hyperlink ref="B26" r:id="rId4" xr:uid="{F69380EC-F02F-3248-8452-C3B242B498C8}"/>
     <hyperlink ref="B30" r:id="rId5" xr:uid="{5CA3156B-9721-3142-A63B-D38C60C3C8F8}"/>
-    <hyperlink ref="E30" r:id="rId6" xr:uid="{450C21B2-311A-4240-9377-2C298317BD5F}"/>
-    <hyperlink ref="E24" r:id="rId7" xr:uid="{F0816AD0-892B-854F-AE84-096906024CA6}"/>
-    <hyperlink ref="E13" r:id="rId8" location="product-offering" xr:uid="{D66F56DF-3275-484E-9EEA-4B8BDCA07065}"/>
-    <hyperlink ref="E41" r:id="rId9" location="product-offering" xr:uid="{6A5722D4-E134-2B4B-9800-B8A5A1C1DB3C}"/>
-    <hyperlink ref="E46" r:id="rId10" xr:uid="{903F7E5A-55BD-8C48-BFA5-F47DC8AE5F40}"/>
-    <hyperlink ref="E45" r:id="rId11" xr:uid="{83BF01B4-6941-0247-9A62-2E8D44ABE10A}"/>
-    <hyperlink ref="E35" r:id="rId12" xr:uid="{DABB9A76-1746-4144-9B1A-570E0C68B3E5}"/>
-    <hyperlink ref="E26" r:id="rId13" xr:uid="{53FAD93A-FDF6-414B-832E-AA3A6DD4C770}"/>
-    <hyperlink ref="E23" r:id="rId14" xr:uid="{69BB09C3-3462-7548-86D1-D168D8CB1CD9}"/>
-    <hyperlink ref="E21" r:id="rId15" xr:uid="{5DF0F16A-35B2-9246-8A86-D188AB376987}"/>
-    <hyperlink ref="E20" r:id="rId16" xr:uid="{6B42F367-F9AE-FE4F-8E9F-CDB10B039F54}"/>
-    <hyperlink ref="E19" r:id="rId17" xr:uid="{F7769EB6-7B3F-3E47-8F5B-6ED3336F5C82}"/>
-    <hyperlink ref="E18" r:id="rId18" xr:uid="{EADAB026-2B3B-794A-9B35-75BBD4FD76B9}"/>
-    <hyperlink ref="E17" r:id="rId19" xr:uid="{7767B94A-6405-A44D-A8A5-C351D5CEDEF2}"/>
-    <hyperlink ref="E47" r:id="rId20" xr:uid="{ABD98ECD-9E4D-3845-A1C1-12987CB34ECF}"/>
+    <hyperlink ref="D30" r:id="rId6" xr:uid="{450C21B2-311A-4240-9377-2C298317BD5F}"/>
+    <hyperlink ref="D24" r:id="rId7" xr:uid="{F0816AD0-892B-854F-AE84-096906024CA6}"/>
+    <hyperlink ref="D13" r:id="rId8" location="product-offering" xr:uid="{D66F56DF-3275-484E-9EEA-4B8BDCA07065}"/>
+    <hyperlink ref="D41" r:id="rId9" location="product-offering" xr:uid="{6A5722D4-E134-2B4B-9800-B8A5A1C1DB3C}"/>
+    <hyperlink ref="D46" r:id="rId10" xr:uid="{903F7E5A-55BD-8C48-BFA5-F47DC8AE5F40}"/>
+    <hyperlink ref="D45" r:id="rId11" xr:uid="{83BF01B4-6941-0247-9A62-2E8D44ABE10A}"/>
+    <hyperlink ref="D35" r:id="rId12" xr:uid="{DABB9A76-1746-4144-9B1A-570E0C68B3E5}"/>
+    <hyperlink ref="D26" r:id="rId13" xr:uid="{53FAD93A-FDF6-414B-832E-AA3A6DD4C770}"/>
+    <hyperlink ref="D23" r:id="rId14" xr:uid="{69BB09C3-3462-7548-86D1-D168D8CB1CD9}"/>
+    <hyperlink ref="D21" r:id="rId15" xr:uid="{5DF0F16A-35B2-9246-8A86-D188AB376987}"/>
+    <hyperlink ref="D20" r:id="rId16" xr:uid="{6B42F367-F9AE-FE4F-8E9F-CDB10B039F54}"/>
+    <hyperlink ref="D19" r:id="rId17" xr:uid="{F7769EB6-7B3F-3E47-8F5B-6ED3336F5C82}"/>
+    <hyperlink ref="D18" r:id="rId18" xr:uid="{EADAB026-2B3B-794A-9B35-75BBD4FD76B9}"/>
+    <hyperlink ref="D17" r:id="rId19" xr:uid="{7767B94A-6405-A44D-A8A5-C351D5CEDEF2}"/>
+    <hyperlink ref="D47" r:id="rId20" xr:uid="{ABD98ECD-9E4D-3845-A1C1-12987CB34ECF}"/>
     <hyperlink ref="B3" r:id="rId21" xr:uid="{B523E380-ACA0-CC46-9C4A-485C9436AE0F}"/>
     <hyperlink ref="B4" r:id="rId22" xr:uid="{4A2BD303-3CD6-E94C-AA35-109B2D987A09}"/>
-    <hyperlink ref="E4" r:id="rId23" xr:uid="{E1A4C7CC-1449-5448-B66B-541A622C23D8}"/>
+    <hyperlink ref="D4" r:id="rId23" xr:uid="{E1A4C7CC-1449-5448-B66B-541A622C23D8}"/>
     <hyperlink ref="B5" r:id="rId24" xr:uid="{BB8F4641-6F97-0143-B12D-9064DBEA8AF1}"/>
-    <hyperlink ref="E5" r:id="rId25" xr:uid="{D108702A-0150-7644-85E0-29DC9C9F9CDF}"/>
+    <hyperlink ref="D5" r:id="rId25" xr:uid="{D108702A-0150-7644-85E0-29DC9C9F9CDF}"/>
     <hyperlink ref="B7" r:id="rId26" xr:uid="{7E983C2B-1DA2-8D40-90CC-312F65BE43CE}"/>
     <hyperlink ref="B13" r:id="rId27" xr:uid="{BEE0900C-1141-7C4A-B8A3-3C8365D5B4FA}"/>
     <hyperlink ref="B17" r:id="rId28" xr:uid="{C3F2217E-3A34-9043-9D19-B5EF9656F8D4}"/>
@@ -2701,24 +2702,29 @@
     <hyperlink ref="B21" r:id="rId31" xr:uid="{F2C036A0-49C8-334A-8C52-3F2F6BDA48EC}"/>
     <hyperlink ref="B23" r:id="rId32" xr:uid="{1F4FB861-7DED-5F4C-9DA4-F4C315E538CC}"/>
     <hyperlink ref="B24" r:id="rId33" xr:uid="{0548D589-09FF-2E4F-9E1D-ACDBBCEF7B3D}"/>
-    <hyperlink ref="E25" r:id="rId34" location="hardware" xr:uid="{2BAAC8D5-10E0-7744-AADD-9DF9E77181D5}"/>
+    <hyperlink ref="D25" r:id="rId34" location="hardware" xr:uid="{2BAAC8D5-10E0-7744-AADD-9DF9E77181D5}"/>
     <hyperlink ref="B29" r:id="rId35" xr:uid="{F31FC16A-D8B0-C54E-AD8B-FE0CCC544018}"/>
-    <hyperlink ref="E29" r:id="rId36" xr:uid="{42AF65D6-F975-4C43-80A2-A74CDF856174}"/>
+    <hyperlink ref="D29" r:id="rId36" xr:uid="{42AF65D6-F975-4C43-80A2-A74CDF856174}"/>
     <hyperlink ref="B31" r:id="rId37" xr:uid="{AE6BDC51-CBE0-2F48-811A-9C4390240F2D}"/>
-    <hyperlink ref="E31" r:id="rId38" xr:uid="{791CE018-9A68-5641-A8E3-FC6C4EC5964D}"/>
+    <hyperlink ref="D31" r:id="rId38" xr:uid="{791CE018-9A68-5641-A8E3-FC6C4EC5964D}"/>
     <hyperlink ref="B34" r:id="rId39" xr:uid="{3113D4AE-E4E5-9C48-AF9B-3F40751AB920}"/>
     <hyperlink ref="B35" r:id="rId40" xr:uid="{61D363F7-3CD7-FA46-8551-C9442F61B077}"/>
     <hyperlink ref="B39" r:id="rId41" xr:uid="{139D6568-3C45-B148-A406-23840EB3F0E6}"/>
     <hyperlink ref="B42" r:id="rId42" xr:uid="{CDA1D95D-F470-6047-98B9-C5312100655D}"/>
     <hyperlink ref="B43" r:id="rId43" xr:uid="{A7E165BF-C250-A440-BAE9-7F98739B885F}"/>
-    <hyperlink ref="E43" r:id="rId44" location="hardware" xr:uid="{06654BE3-F15A-A34C-802C-AFBD70AB119C}"/>
+    <hyperlink ref="D43" r:id="rId44" location="hardware" xr:uid="{06654BE3-F15A-A34C-802C-AFBD70AB119C}"/>
     <hyperlink ref="B45" r:id="rId45" xr:uid="{99EF6A8F-E2F3-4F48-8F07-CAA3D17C760C}"/>
     <hyperlink ref="B46" r:id="rId46" xr:uid="{66E05957-9A35-7C40-A987-C6054B222313}"/>
     <hyperlink ref="B47" r:id="rId47" xr:uid="{7202F1B2-4E39-084E-9E14-EABAF8C6C2DB}"/>
     <hyperlink ref="B48" r:id="rId48" xr:uid="{C4E25341-C554-E743-8CBA-276D146F5874}"/>
-    <hyperlink ref="E48" r:id="rId49" xr:uid="{1D183AA4-ABDD-A846-B415-51F946E14724}"/>
+    <hyperlink ref="D48" r:id="rId49" xr:uid="{1D183AA4-ABDD-A846-B415-51F946E14724}"/>
     <hyperlink ref="B49" r:id="rId50" xr:uid="{A0363C17-9D8F-C543-9E08-EE37DE3D5BD7}"/>
-    <hyperlink ref="E49" r:id="rId51" xr:uid="{E1DA5D50-2EC4-1C43-B465-23311234B42A}"/>
+    <hyperlink ref="D49" r:id="rId51" xr:uid="{E1DA5D50-2EC4-1C43-B465-23311234B42A}"/>
+    <hyperlink ref="B22" r:id="rId52" xr:uid="{5CF21884-06E7-DA42-A6CB-7CEA69ED12FB}"/>
+    <hyperlink ref="D22" r:id="rId53" xr:uid="{2193DC12-A42F-4A4B-A26F-8A6F0D43EAAD}"/>
+    <hyperlink ref="D36" r:id="rId54" xr:uid="{61BE7470-2D42-2349-B0D1-42445CDC87A2}"/>
+    <hyperlink ref="D44" r:id="rId55" xr:uid="{179D6384-8E00-2D47-8744-B69473AE5E29}"/>
+    <hyperlink ref="D33" r:id="rId56" location="hardware-installation" xr:uid="{870B4EE4-A691-F343-85E3-9CD4A18CD4F9}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2734,7 +2740,7 @@
   <sheetData>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
   </sheetData>
@@ -2767,199 +2773,199 @@
         <v>284</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="14">
+    <row r="2" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="12">
         <v>2</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="14">
+      <c r="E2" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="12">
         <v>3</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="E3" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="14">
+      <c r="E3" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="12">
         <v>4</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="E4" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="14">
+      <c r="E4" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="12">
         <v>5</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="E5" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="14">
+      <c r="E5" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="12">
         <v>6</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="E6" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="14">
+      <c r="E6" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="12">
         <v>7</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="E7" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="14">
+      <c r="E7" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="12">
         <v>8</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="E8" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="14">
+      <c r="E8" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="12">
         <v>9</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="E9" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="14">
+      <c r="E9" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="12">
         <v>10</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="E10" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="14">
+      <c r="E10" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="12">
         <v>11</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="E11" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="14">
-        <v>12</v>
-      </c>
-      <c r="B12" s="14" t="s">
+      <c r="E11" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="12">
+        <v>12</v>
+      </c>
+      <c r="B12" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="E12" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="14">
+      <c r="E12" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="12">
         <v>31</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="E13" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="14">
+      <c r="E13" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="12">
         <v>33</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="E14" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="14">
+      <c r="E14" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="12">
         <v>34</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="13" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3075,7 +3081,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8367F40A-2872-F249-9EF5-B63EF25E34CB}">
-  <dimension ref="A1:E104"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.5" customWidth="1"/>
@@ -3241,14 +3247,14 @@
         <v>349</v>
       </c>
     </row>
-    <row r="15" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="16">
+    <row r="15" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="14">
         <v>47</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="15" t="s">
         <v>348</v>
       </c>
     </row>
@@ -3615,516 +3621,505 @@
         <v>344</v>
       </c>
     </row>
-    <row r="49" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="13">
+    <row r="49" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="11">
         <v>22</v>
       </c>
-      <c r="B49" s="13" t="s">
+      <c r="B49" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="E49" s="18" t="s">
+      <c r="E49" s="16" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="50" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="13">
+    <row r="50" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="11">
         <v>23</v>
       </c>
-      <c r="B50" s="13" t="s">
+      <c r="B50" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="E50" s="18" t="s">
+      <c r="E50" s="16" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="51" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="13">
+    <row r="51" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="11">
         <v>24</v>
       </c>
-      <c r="B51" s="18" t="s">
+      <c r="B51" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="E51" s="18" t="s">
+      <c r="E51" s="16" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="52" spans="1:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="19">
+    <row r="52" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="17">
         <v>42</v>
       </c>
-      <c r="B52" s="19" t="s">
+      <c r="B52" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="E52" s="20" t="s">
+      <c r="E52" s="18" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="53" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="13">
+    <row r="53" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="11">
         <v>26</v>
       </c>
-      <c r="B53" s="13" t="s">
+      <c r="B53" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="E53" s="18" t="s">
+      <c r="E53" s="16" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="54" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="13">
+    <row r="54" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="11">
         <v>28</v>
       </c>
-      <c r="B54" s="18" t="s">
+      <c r="B54" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="E54" s="18" t="s">
+      <c r="E54" s="16" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="55" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="13">
+    <row r="55" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="11">
         <v>29</v>
       </c>
-      <c r="B55" s="13" t="s">
+      <c r="B55" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="E55" s="18" t="s">
+      <c r="E55" s="16" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="56" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="16">
+    <row r="56" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="14">
         <v>48</v>
       </c>
-      <c r="B56" s="16" t="s">
+      <c r="B56" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="E56" s="17" t="s">
+      <c r="E56" s="15" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="57" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="16">
+    <row r="57" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="14">
         <v>14</v>
       </c>
-      <c r="B57" s="16" t="s">
+      <c r="B57" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="E57" s="17" t="s">
+      <c r="E57" s="15" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="58" spans="1:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="19">
+    <row r="58" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="17">
         <v>37</v>
       </c>
-      <c r="B58" s="19" t="s">
+      <c r="B58" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="E58" s="20" t="s">
+      <c r="E58" s="18" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="59" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="16">
+    <row r="59" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="14">
         <v>81</v>
       </c>
-      <c r="B59" s="16" t="s">
+      <c r="B59" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="E59" s="17" t="s">
+      <c r="E59" s="15" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="60" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="16">
+    <row r="60" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="14">
         <v>75</v>
       </c>
-      <c r="B60" s="16" t="s">
+      <c r="B60" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="E60" s="17" t="s">
+      <c r="E60" s="15" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="61" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="16">
+    <row r="61" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="14">
         <v>66</v>
       </c>
-      <c r="B61" s="16" t="s">
+      <c r="B61" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="E61" s="17" t="s">
+      <c r="E61" s="15" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="62" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="16">
+    <row r="62" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="14">
         <v>67</v>
       </c>
-      <c r="B62" s="16" t="s">
+      <c r="B62" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="E62" s="17" t="s">
+      <c r="E62" s="15" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="63" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="16">
+    <row r="63" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="14">
         <v>70</v>
       </c>
-      <c r="B63" s="16" t="s">
+      <c r="B63" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="E63" s="17" t="s">
+      <c r="E63" s="15" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="64" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="16">
+    <row r="64" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="14">
         <v>71</v>
       </c>
-      <c r="B64" s="16" t="s">
+      <c r="B64" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="E64" s="17" t="s">
+      <c r="E64" s="15" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="65" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="16">
+    <row r="65" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="14">
         <v>54</v>
       </c>
-      <c r="B65" s="16" t="s">
+      <c r="B65" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="E65" s="17" t="s">
+      <c r="E65" s="15" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="66" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="16">
+    <row r="66" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="14">
         <v>59</v>
       </c>
-      <c r="B66" s="16" t="s">
+      <c r="B66" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="E66" s="17" t="s">
+      <c r="E66" s="15" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="67" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="16">
+    <row r="67" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="14">
         <v>56</v>
       </c>
-      <c r="B67" s="16" t="s">
+      <c r="B67" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="E67" s="17" t="s">
+      <c r="E67" s="15" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="68" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="16">
+    <row r="68" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="14">
         <v>49</v>
       </c>
-      <c r="B68" s="16" t="s">
+      <c r="B68" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="E68" s="17" t="s">
+      <c r="E68" s="15" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="69" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="13">
+    <row r="69" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="11">
         <v>27</v>
       </c>
-      <c r="B69" s="13" t="s">
+      <c r="B69" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="E69" s="18" t="s">
+      <c r="E69" s="16" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="70" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="16">
+    <row r="70" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="14">
         <v>30</v>
       </c>
-      <c r="B70" s="16" t="s">
+      <c r="B70" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="E70" s="17" t="s">
+      <c r="E70" s="15" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="71" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="16">
+    <row r="71" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="14">
         <v>44</v>
       </c>
-      <c r="B71" s="16" t="s">
+      <c r="B71" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="E71" s="17" t="s">
+      <c r="E71" s="15" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="72" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="16">
+    <row r="72" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="14">
         <v>45</v>
       </c>
-      <c r="B72" s="16" t="s">
+      <c r="B72" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="E72" s="17" t="s">
+      <c r="E72" s="15" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="73" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="16">
+    <row r="73" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="14">
         <v>46</v>
       </c>
-      <c r="B73" s="16" t="s">
+      <c r="B73" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="E73" s="17" t="s">
+      <c r="E73" s="15" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="74" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="16">
+    <row r="74" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="14">
         <v>52</v>
       </c>
-      <c r="B74" s="16" t="s">
+      <c r="B74" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="E74" s="17" t="s">
+      <c r="E74" s="15" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="75" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="16">
+    <row r="75" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="14">
         <v>55</v>
       </c>
-      <c r="B75" s="16" t="s">
+      <c r="B75" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="E75" s="17" t="s">
+      <c r="E75" s="15" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="76" spans="1:5" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="16">
+    <row r="76" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A76" s="14">
         <v>65</v>
       </c>
-      <c r="B76" s="16" t="s">
+      <c r="B76" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="E76" s="17" t="s">
+      <c r="E76" s="15" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="77" spans="1:5" s="19" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="19">
+    <row r="77" spans="1:5" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="17">
         <v>69</v>
       </c>
-      <c r="B77" s="19" t="s">
+      <c r="B77" s="17" t="s">
         <v>171</v>
       </c>
-      <c r="E77" s="20" t="s">
+      <c r="E77" s="18" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="78" spans="1:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="19">
+    <row r="78" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="17">
         <v>74</v>
       </c>
-      <c r="B78" s="19" t="s">
+      <c r="B78" s="17" t="s">
         <v>176</v>
       </c>
-      <c r="E78" s="20" t="s">
+      <c r="E78" s="18" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="79" spans="1:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="19">
+    <row r="79" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="17">
         <v>32</v>
       </c>
-      <c r="B79" s="19" t="s">
+      <c r="B79" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="E79" s="20" t="s">
+      <c r="E79" s="18" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="80" spans="1:5" s="24" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="E80" s="7"/>
-    </row>
-    <row r="81" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B80" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="E80" s="21" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="81" spans="2:5" s="20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B81" s="21" t="s">
-        <v>98</v>
-      </c>
-      <c r="E81" s="23" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="82" spans="2:5" s="22" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B82" s="22" t="s">
         <v>180</v>
       </c>
-      <c r="E82" s="23" t="s">
+      <c r="E81" s="21" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="83" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B82" s="21" t="s">
+        <v>163</v>
+      </c>
+      <c r="E82" s="21" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="83" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B83" s="21" t="s">
-        <v>163</v>
-      </c>
-      <c r="E83" s="23" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="84" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
+        <v>178</v>
+      </c>
+      <c r="E83" s="21" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="84" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B84" s="21" t="s">
-        <v>178</v>
-      </c>
-      <c r="E84" s="23" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="85" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
+        <v>179</v>
+      </c>
+      <c r="E84" s="21" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="85" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B85" s="21" t="s">
-        <v>179</v>
-      </c>
-      <c r="E85" s="23" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="86" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
+        <v>181</v>
+      </c>
+      <c r="E85" s="21" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="86" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B86" s="21" t="s">
-        <v>181</v>
-      </c>
-      <c r="E86" s="23" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="87" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+      <c r="E86" s="21" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="87" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B87" s="21" t="s">
-        <v>182</v>
-      </c>
-      <c r="E87" s="23" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="88" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
+        <v>160</v>
+      </c>
+      <c r="E87" s="21" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="88" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B88" s="21" t="s">
-        <v>160</v>
-      </c>
-      <c r="E88" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="E88" s="21" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="89" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B89" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="E89" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="E89" s="21" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="90" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B90" s="21" t="s">
-        <v>155</v>
-      </c>
-      <c r="E90" s="23" t="s">
+        <v>135</v>
+      </c>
+      <c r="E90" s="21" t="s">
         <v>404</v>
       </c>
     </row>
-    <row r="91" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B91" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="E91" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="E91" s="21" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="92" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B92" s="21" t="s">
+        <v>165</v>
+      </c>
+      <c r="E92" s="21" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="92" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B92" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="E92" s="23" t="s">
+    <row r="93" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B93" s="21" t="s">
+        <v>166</v>
+      </c>
+      <c r="E93" s="21" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="93" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B93" s="21" t="s">
-        <v>165</v>
-      </c>
-      <c r="E93" s="23" t="s">
+    <row r="94" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B94" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="E94" s="21" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="94" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B94" s="21" t="s">
-        <v>166</v>
-      </c>
-      <c r="E94" s="23" t="s">
+    <row r="95" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B95" s="21" t="s">
+        <v>159</v>
+      </c>
+      <c r="E95" s="21" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="95" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B95" s="21" t="s">
-        <v>152</v>
-      </c>
-      <c r="E95" s="23" t="s">
+    <row r="96" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B96" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="E96" s="21" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="97" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B97" s="21" t="s">
+        <v>164</v>
+      </c>
+      <c r="E97" s="21" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="98" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B98" s="21" t="s">
+        <v>123</v>
+      </c>
+      <c r="E98" s="21" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="99" spans="2:5" s="19" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B99" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="E99" s="21" t="s">
         <v>409</v>
-      </c>
-    </row>
-    <row r="96" spans="2:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B96" s="21" t="s">
-        <v>159</v>
-      </c>
-      <c r="E96" s="23" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B97" s="21" t="s">
-        <v>162</v>
-      </c>
-      <c r="E97" s="23" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B98" s="21" t="s">
-        <v>164</v>
-      </c>
-      <c r="E98" s="23" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B99" s="21" t="s">
-        <v>123</v>
-      </c>
-      <c r="E99" s="23" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B100" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="E100" s="23" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A104" t="s">
-        <v>415</v>
-      </c>
-      <c r="B104" t="s">
-        <v>400</v>
       </c>
     </row>
   </sheetData>
@@ -4213,26 +4208,46 @@
     <hyperlink ref="E78" r:id="rId82" xr:uid="{A5E9C8AD-4B4D-B343-8E89-F55BA0E21068}"/>
     <hyperlink ref="E77" r:id="rId83" xr:uid="{35582EA3-B7FA-014E-8D16-0237FB2358D4}"/>
     <hyperlink ref="E79" r:id="rId84" xr:uid="{0107F09A-5542-A848-A1D5-15B750AB1291}"/>
-    <hyperlink ref="E83" r:id="rId85" xr:uid="{67F6EBBE-F2AE-B141-A792-EE16B731B2F2}"/>
-    <hyperlink ref="E82" r:id="rId86" xr:uid="{81FAD121-2F1D-1D40-B9A2-6B59A51C3611}"/>
-    <hyperlink ref="E81" r:id="rId87" xr:uid="{8A8295AB-D568-544A-98DB-19621A0252EB}"/>
-    <hyperlink ref="E87" r:id="rId88" xr:uid="{C195B8E0-C7F4-4741-B07A-46E007FFA1A1}"/>
-    <hyperlink ref="E86" r:id="rId89" xr:uid="{70CE0B20-FC6F-0A40-A990-27F52309E366}"/>
-    <hyperlink ref="E85" r:id="rId90" xr:uid="{54855452-473D-464C-8EAF-5F6C3B8690AB}"/>
-    <hyperlink ref="E84" r:id="rId91" xr:uid="{235F28B2-676F-3D48-955D-7659FFAFE7BD}"/>
-    <hyperlink ref="E88" r:id="rId92" xr:uid="{2A2F225E-21DB-C94B-9CA3-642E367C0295}"/>
-    <hyperlink ref="E89" r:id="rId93" xr:uid="{DA0F23EC-5831-3244-BB06-EE603014E78F}"/>
-    <hyperlink ref="E90" r:id="rId94" xr:uid="{86F9C7E7-3D01-2D43-8118-11C3EC8CB5B8}"/>
-    <hyperlink ref="E91" r:id="rId95" xr:uid="{15A6E8F4-559C-584F-8A2A-BA851AE5BD8B}"/>
-    <hyperlink ref="E92" r:id="rId96" xr:uid="{4CFA57D0-7372-2345-AD38-C82A7A432CA9}"/>
-    <hyperlink ref="E93" r:id="rId97" xr:uid="{84A9F0AF-5BEF-8343-905C-407A7C297750}"/>
-    <hyperlink ref="E94" r:id="rId98" xr:uid="{FDDFDE82-6A12-D343-836D-73A841098D71}"/>
-    <hyperlink ref="E97" r:id="rId99" xr:uid="{88AB027B-0BFF-C445-89DF-C73C5C9C75AB}"/>
-    <hyperlink ref="E98" r:id="rId100" xr:uid="{9364D6E8-87E0-B641-8C88-40FD581EFDC0}"/>
-    <hyperlink ref="E99" r:id="rId101" xr:uid="{577EDBE6-C761-D04E-B177-9BD4A5397CE7}"/>
-    <hyperlink ref="E100" r:id="rId102" xr:uid="{705C30E7-FB74-634C-B831-3A980E832B2B}"/>
-    <hyperlink ref="E96" r:id="rId103" xr:uid="{27AE31CC-AB5B-A842-8867-D7C5AFF89138}"/>
-    <hyperlink ref="E95" r:id="rId104" xr:uid="{282EFEF8-AAE3-3A49-A05F-168C5AF67755}"/>
+    <hyperlink ref="E82" r:id="rId85" xr:uid="{67F6EBBE-F2AE-B141-A792-EE16B731B2F2}"/>
+    <hyperlink ref="E81" r:id="rId86" xr:uid="{81FAD121-2F1D-1D40-B9A2-6B59A51C3611}"/>
+    <hyperlink ref="E80" r:id="rId87" xr:uid="{8A8295AB-D568-544A-98DB-19621A0252EB}"/>
+    <hyperlink ref="E86" r:id="rId88" xr:uid="{C195B8E0-C7F4-4741-B07A-46E007FFA1A1}"/>
+    <hyperlink ref="E85" r:id="rId89" xr:uid="{70CE0B20-FC6F-0A40-A990-27F52309E366}"/>
+    <hyperlink ref="E84" r:id="rId90" xr:uid="{54855452-473D-464C-8EAF-5F6C3B8690AB}"/>
+    <hyperlink ref="E83" r:id="rId91" xr:uid="{235F28B2-676F-3D48-955D-7659FFAFE7BD}"/>
+    <hyperlink ref="E87" r:id="rId92" xr:uid="{2A2F225E-21DB-C94B-9CA3-642E367C0295}"/>
+    <hyperlink ref="E88" r:id="rId93" xr:uid="{DA0F23EC-5831-3244-BB06-EE603014E78F}"/>
+    <hyperlink ref="E89" r:id="rId94" xr:uid="{86F9C7E7-3D01-2D43-8118-11C3EC8CB5B8}"/>
+    <hyperlink ref="E90" r:id="rId95" xr:uid="{15A6E8F4-559C-584F-8A2A-BA851AE5BD8B}"/>
+    <hyperlink ref="E91" r:id="rId96" xr:uid="{4CFA57D0-7372-2345-AD38-C82A7A432CA9}"/>
+    <hyperlink ref="E92" r:id="rId97" xr:uid="{84A9F0AF-5BEF-8343-905C-407A7C297750}"/>
+    <hyperlink ref="E93" r:id="rId98" xr:uid="{FDDFDE82-6A12-D343-836D-73A841098D71}"/>
+    <hyperlink ref="E96" r:id="rId99" xr:uid="{88AB027B-0BFF-C445-89DF-C73C5C9C75AB}"/>
+    <hyperlink ref="E97" r:id="rId100" xr:uid="{9364D6E8-87E0-B641-8C88-40FD581EFDC0}"/>
+    <hyperlink ref="E98" r:id="rId101" xr:uid="{577EDBE6-C761-D04E-B177-9BD4A5397CE7}"/>
+    <hyperlink ref="E99" r:id="rId102" xr:uid="{705C30E7-FB74-634C-B831-3A980E832B2B}"/>
+    <hyperlink ref="E95" r:id="rId103" xr:uid="{27AE31CC-AB5B-A842-8867-D7C5AFF89138}"/>
+    <hyperlink ref="E94" r:id="rId104" xr:uid="{282EFEF8-AAE3-3A49-A05F-168C5AF67755}"/>
+    <hyperlink ref="B80" r:id="rId105" xr:uid="{026E541D-261B-E048-A181-5EDD64375248}"/>
+    <hyperlink ref="B81" r:id="rId106" xr:uid="{3DFD8E7E-2E7E-6B4B-8632-C5F2F8CD4EA6}"/>
+    <hyperlink ref="B82" r:id="rId107" xr:uid="{77327480-16A7-EF42-9409-D70F37481FD0}"/>
+    <hyperlink ref="B83" r:id="rId108" xr:uid="{573BE0C9-0621-A549-9AD7-6D91D2B7E306}"/>
+    <hyperlink ref="B84" r:id="rId109" xr:uid="{051202F1-79F5-B144-A7FF-B3FE091A2CC5}"/>
+    <hyperlink ref="B85" r:id="rId110" xr:uid="{C0BA4C15-C07E-CE48-A1D2-0CD18C21C6BC}"/>
+    <hyperlink ref="B86" r:id="rId111" xr:uid="{163DBF5E-6024-8A43-85DB-41FB13F50935}"/>
+    <hyperlink ref="B87" r:id="rId112" xr:uid="{99D0C494-2FE9-524A-9AC0-796E8B87C5C4}"/>
+    <hyperlink ref="B88" r:id="rId113" xr:uid="{131ACD98-7D38-E74D-96A5-7EF51E0D4B35}"/>
+    <hyperlink ref="B89" r:id="rId114" xr:uid="{8A822B45-493E-AD44-8FA0-ADE035A99ED4}"/>
+    <hyperlink ref="B90" r:id="rId115" xr:uid="{A797F28F-88FE-6043-AAB1-66BC04E9DC95}"/>
+    <hyperlink ref="B91" r:id="rId116" xr:uid="{D21AA6C7-6553-7445-AAB4-7BAA3EF4861A}"/>
+    <hyperlink ref="B92" r:id="rId117" xr:uid="{0C53D11C-96C1-2F43-B9C0-695657BB26FE}"/>
+    <hyperlink ref="B93" r:id="rId118" xr:uid="{5F571A20-5F7C-114D-8A79-66ECAA9B7C0F}"/>
+    <hyperlink ref="B94" r:id="rId119" xr:uid="{A15350D1-6C75-DB47-848A-A6F6B234F3BB}"/>
+    <hyperlink ref="B95" r:id="rId120" xr:uid="{1F495420-ECF0-0540-AE23-A10610447599}"/>
+    <hyperlink ref="B96" r:id="rId121" xr:uid="{B2B10F1D-99D9-6045-BCC8-EDE334DDED29}"/>
+    <hyperlink ref="B97" r:id="rId122" xr:uid="{A9A4B604-6603-E040-A6CC-F35D30844B24}"/>
+    <hyperlink ref="B98" r:id="rId123" xr:uid="{42E5006F-35FC-0949-939D-C36A1F194D75}"/>
+    <hyperlink ref="B99" r:id="rId124" xr:uid="{A17716DF-0971-944B-9AAB-B5476A2E226A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>